<commit_message>
final dataset achieved for turker training!!!
</commit_message>
<xml_diff>
--- a/src/dataset_comparison_scripts/statistical_analysis/prerana_analysis/final_adjudicated_set - Final_adjudicated set.xlsx
+++ b/src/dataset_comparison_scripts/statistical_analysis/prerana_analysis/final_adjudicated_set - Final_adjudicated set.xlsx
@@ -977,7 +977,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -5257,51 +5257,69 @@
         <v>126</v>
       </c>
     </row>
-    <row r="86" hidden="1">
-      <c r="A86" s="4" t="s">
-        <v>127</v>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>george conway urges trump to resign over aborted iran strike</t>
+        </is>
       </c>
       <c r="B86" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D86" s="5">
-        <v>46054.0</v>
+        <v>3</v>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>majority_accept</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
       </c>
       <c r="E86" s="4">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F86" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="G86" s="4">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="H86" s="4">
-        <v>0.666666666666666</v>
-      </c>
-      <c r="I86" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J86" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K86" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="L86" s="4" t="s">
-        <v>51</v>
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>bandwagon</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>persuasive propaganda</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="inlineStr">
+        <is>
+          <t>whose judgment no serious, intelligent person trusts</t>
+        </is>
+      </c>
+      <c r="L86" s="4" t="inlineStr">
+        <is>
+          <t>Aarush</t>
+        </is>
       </c>
       <c r="M86" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="N86" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="O86" s="4" t="s">
-        <v>128</v>
+        <v>1</v>
+      </c>
+      <c r="N86" s="4" t="inlineStr">
+        <is>
+          <t>Aarush</t>
+        </is>
+      </c>
+      <c r="O86" s="4" t="inlineStr">
+        <is>
+          <t>whose judgment no serious, intelligent person trusts</t>
+        </is>
       </c>
     </row>
     <row r="87" hidden="1">
@@ -5330,25 +5348,25 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="K87" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L87" s="4" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="M87" s="4">
         <v>1.0</v>
       </c>
       <c r="N87" s="4" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="O87" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="88" hidden="1">
@@ -5383,7 +5401,7 @@
         <v>18</v>
       </c>
       <c r="K88" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L88" s="4" t="s">
         <v>29</v>
@@ -5395,12 +5413,12 @@
         <v>29</v>
       </c>
       <c r="O88" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="89" hidden="1">
       <c r="A89" s="4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B89" s="4">
         <v>0.0</v>
@@ -5424,13 +5442,13 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="J89" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K89" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L89" s="4" t="s">
         <v>29</v>
@@ -5442,323 +5460,323 @@
         <v>29</v>
       </c>
       <c r="O89" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="90" hidden="1">
+      <c r="A90" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B90" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D90" s="5">
+        <v>46054.0</v>
+      </c>
+      <c r="E90" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="F90" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="G90" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="H90" s="4">
+        <v>0.666666666666666</v>
+      </c>
+      <c r="I90" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J90" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K90" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="7" t="s">
+      <c r="L90" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="M90" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="N90" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="O90" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B90" s="7">
+      <c r="B91" s="7">
         <v>0.0</v>
       </c>
-      <c r="C90" s="7" t="s">
+      <c r="C91" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D90" s="7" t="s">
+      <c r="D91" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E90" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="F90" s="7">
+      <c r="E91" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F91" s="7">
         <v>0.0</v>
       </c>
-      <c r="G90" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="H90" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="I90" s="7" t="s">
+      <c r="G91" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="H91" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="I91" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J90" s="7" t="s">
+      <c r="J91" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="K90" s="7" t="s">
+      <c r="K91" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="L90" s="7" t="s">
+      <c r="L91" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M90" s="7">
+      <c r="M91" s="7">
         <v>2.0</v>
       </c>
-      <c r="N90" s="7" t="s">
+      <c r="N91" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="O90" s="7" t="s">
+      <c r="O91" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="P90" s="8"/>
-      <c r="Q90" s="8"/>
-      <c r="R90" s="8"/>
-      <c r="S90" s="8"/>
-      <c r="T90" s="8"/>
-      <c r="U90" s="8"/>
-      <c r="V90" s="8"/>
-      <c r="W90" s="8"/>
-      <c r="X90" s="8"/>
-      <c r="Y90" s="8"/>
-      <c r="Z90" s="8"/>
-    </row>
-    <row r="91" hidden="1">
-      <c r="A91" s="4" t="s">
+      <c r="P91" s="8"/>
+      <c r="Q91" s="8"/>
+      <c r="R91" s="8"/>
+      <c r="S91" s="8"/>
+      <c r="T91" s="8"/>
+      <c r="U91" s="8"/>
+      <c r="V91" s="8"/>
+      <c r="W91" s="8"/>
+      <c r="X91" s="8"/>
+      <c r="Y91" s="8"/>
+      <c r="Z91" s="8"/>
+    </row>
+    <row r="92" hidden="1">
+      <c r="A92" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B91" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="C91" s="4" t="s">
+      <c r="B92" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C92" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D91" s="5">
+      <c r="D92" s="5">
         <v>46054.0</v>
       </c>
-      <c r="E91" s="4">
+      <c r="E92" s="4">
         <v>2.0</v>
       </c>
-      <c r="F91" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="G91" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="H91" s="4">
+      <c r="F92" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="G92" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="H92" s="4">
         <v>0.666666666666666</v>
       </c>
-      <c r="I91" s="4" t="s">
+      <c r="I92" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="J91" s="4" t="s">
+      <c r="J92" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K91" s="4" t="s">
+      <c r="K92" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="L91" s="4" t="s">
+      <c r="L92" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M91" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="N91" s="4" t="s">
+      <c r="M92" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="N92" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="O91" s="4" t="s">
+      <c r="O92" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="7" t="s">
+    <row r="93">
+      <c r="A93" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B92" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="C92" s="7" t="s">
+      <c r="B93" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="C93" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D92" s="7" t="s">
+      <c r="D93" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E92" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="F92" s="7">
+      <c r="E93" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F93" s="7">
         <v>0.0</v>
       </c>
-      <c r="G92" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="H92" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="I92" s="7" t="s">
+      <c r="G93" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="H93" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="I93" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J92" s="7" t="s">
+      <c r="J93" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="K92" s="7" t="s">
+      <c r="K93" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="L92" s="7" t="s">
+      <c r="L93" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="M92" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="N92" s="7" t="s">
+      <c r="M93" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="N93" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="O92" s="7" t="s">
+      <c r="O93" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="P92" s="8"/>
-      <c r="Q92" s="8"/>
-      <c r="R92" s="8"/>
-      <c r="S92" s="8"/>
-      <c r="T92" s="8"/>
-      <c r="U92" s="8"/>
-      <c r="V92" s="8"/>
-      <c r="W92" s="8"/>
-      <c r="X92" s="8"/>
-      <c r="Y92" s="8"/>
-      <c r="Z92" s="8"/>
-    </row>
-    <row r="93" hidden="1">
-      <c r="A93" s="4" t="s">
+      <c r="P93" s="8"/>
+      <c r="Q93" s="8"/>
+      <c r="R93" s="8"/>
+      <c r="S93" s="8"/>
+      <c r="T93" s="8"/>
+      <c r="U93" s="8"/>
+      <c r="V93" s="8"/>
+      <c r="W93" s="8"/>
+      <c r="X93" s="8"/>
+      <c r="Y93" s="8"/>
+      <c r="Z93" s="8"/>
+    </row>
+    <row r="94" hidden="1">
+      <c r="A94" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B93" s="4">
+      <c r="B94" s="4">
         <v>0.0</v>
       </c>
-      <c r="C93" s="4" t="s">
+      <c r="C94" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D93" s="5">
+      <c r="D94" s="5">
         <v>46054.0</v>
       </c>
-      <c r="E93" s="4">
+      <c r="E94" s="4">
         <v>2.0</v>
       </c>
-      <c r="F93" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="G93" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="H93" s="4">
+      <c r="F94" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="G94" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="H94" s="4">
         <v>0.666666666666666</v>
       </c>
-      <c r="I93" s="4" t="s">
+      <c r="I94" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J93" s="4" t="s">
+      <c r="J94" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K93" s="4" t="s">
+      <c r="K94" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="L93" s="4" t="s">
+      <c r="L94" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M93" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="N93" s="4" t="s">
+      <c r="M94" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="N94" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="O93" s="4" t="s">
+      <c r="O94" s="4" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="7" t="s">
+    <row r="95">
+      <c r="A95" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B94" s="7">
+      <c r="B95" s="7">
         <v>0.0</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="C95" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D94" s="7" t="s">
+      <c r="D95" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E94" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="F94" s="7">
+      <c r="E95" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F95" s="7">
         <v>0.0</v>
       </c>
-      <c r="G94" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="H94" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="I94" s="7" t="s">
+      <c r="G95" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="H95" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="I95" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J94" s="7" t="s">
+      <c r="J95" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="K94" s="7" t="s">
+      <c r="K95" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="L94" s="7" t="s">
+      <c r="L95" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M94" s="7">
+      <c r="M95" s="7">
         <v>2.0</v>
       </c>
-      <c r="N94" s="7" t="s">
+      <c r="N95" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="O94" s="7" t="s">
+      <c r="O95" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="P94" s="8"/>
-      <c r="Q94" s="8"/>
-      <c r="R94" s="8"/>
-      <c r="S94" s="8"/>
-      <c r="T94" s="8"/>
-      <c r="U94" s="8"/>
-      <c r="V94" s="8"/>
-      <c r="W94" s="8"/>
-      <c r="X94" s="8"/>
-      <c r="Y94" s="8"/>
-      <c r="Z94" s="8"/>
-    </row>
-    <row r="95" hidden="1">
-      <c r="A95" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="B95" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D95" s="5">
-        <v>46054.0</v>
-      </c>
-      <c r="E95" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="F95" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="G95" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="H95" s="4">
-        <v>0.666666666666666</v>
-      </c>
-      <c r="I95" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J95" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K95" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="L95" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="M95" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="N95" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="O95" s="4" t="s">
-        <v>136</v>
-      </c>
+      <c r="P95" s="8"/>
+      <c r="Q95" s="8"/>
+      <c r="R95" s="8"/>
+      <c r="S95" s="8"/>
+      <c r="T95" s="8"/>
+      <c r="U95" s="8"/>
+      <c r="V95" s="8"/>
+      <c r="W95" s="8"/>
+      <c r="X95" s="8"/>
+      <c r="Y95" s="8"/>
+      <c r="Z95" s="8"/>
     </row>
     <row r="96" hidden="1">
       <c r="A96" s="4" t="s">
@@ -5786,13 +5804,13 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="J96" s="4" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="K96" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L96" s="4" t="s">
         <v>29</v>
@@ -5804,218 +5822,218 @@
         <v>29</v>
       </c>
       <c r="O96" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="97" hidden="1">
+      <c r="A97" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B97" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D97" s="5">
+        <v>46054.0</v>
+      </c>
+      <c r="E97" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="F97" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="G97" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="H97" s="4">
+        <v>0.666666666666666</v>
+      </c>
+      <c r="I97" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J97" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K97" s="4" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="7" t="s">
+      <c r="L97" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="M97" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="N97" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="O97" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B97" s="7">
+      <c r="B98" s="7">
         <v>2.0</v>
       </c>
-      <c r="C97" s="7" t="s">
+      <c r="C98" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D97" s="7" t="s">
+      <c r="D98" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E97" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="F97" s="7">
+      <c r="E98" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F98" s="7">
         <v>0.0</v>
       </c>
-      <c r="G97" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="H97" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="I97" s="7" t="s">
+      <c r="G98" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="H98" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="I98" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="J97" s="7" t="s">
+      <c r="J98" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="K97" s="7" t="s">
+      <c r="K98" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="L97" s="7" t="s">
+      <c r="L98" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="M97" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="N97" s="7" t="s">
+      <c r="M98" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="N98" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="O97" s="7" t="s">
+      <c r="O98" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="P97" s="8"/>
-      <c r="Q97" s="8"/>
-      <c r="R97" s="8"/>
-      <c r="S97" s="8"/>
-      <c r="T97" s="8"/>
-      <c r="U97" s="8"/>
-      <c r="V97" s="8"/>
-      <c r="W97" s="8"/>
-      <c r="X97" s="8"/>
-      <c r="Y97" s="8"/>
-      <c r="Z97" s="8"/>
-    </row>
-    <row r="98" hidden="1">
-      <c r="A98" s="4" t="s">
+      <c r="P98" s="8"/>
+      <c r="Q98" s="8"/>
+      <c r="R98" s="8"/>
+      <c r="S98" s="8"/>
+      <c r="T98" s="8"/>
+      <c r="U98" s="8"/>
+      <c r="V98" s="8"/>
+      <c r="W98" s="8"/>
+      <c r="X98" s="8"/>
+      <c r="Y98" s="8"/>
+      <c r="Z98" s="8"/>
+    </row>
+    <row r="99" hidden="1">
+      <c r="A99" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B98" s="4">
+      <c r="B99" s="4">
         <v>2.0</v>
       </c>
-      <c r="C98" s="4" t="s">
+      <c r="C99" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D98" s="5">
+      <c r="D99" s="5">
         <v>46054.0</v>
       </c>
-      <c r="E98" s="4">
+      <c r="E99" s="4">
         <v>2.0</v>
       </c>
-      <c r="F98" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="G98" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="H98" s="4">
+      <c r="F99" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="G99" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="H99" s="4">
         <v>0.666666666666666</v>
       </c>
-      <c r="I98" s="4" t="s">
+      <c r="I99" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="J98" s="4" t="s">
+      <c r="J99" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K98" s="4" t="s">
+      <c r="K99" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="L98" s="4" t="s">
+      <c r="L99" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M98" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="N98" s="4" t="s">
+      <c r="M99" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="N99" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="O98" s="4" t="s">
+      <c r="O99" s="4" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="7" t="s">
+    <row r="100">
+      <c r="A100" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B99" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="C99" s="7" t="s">
+      <c r="B100" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="C100" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D99" s="7" t="s">
+      <c r="D100" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E99" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="F99" s="7">
+      <c r="E100" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F100" s="7">
         <v>0.0</v>
       </c>
-      <c r="G99" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="H99" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="I99" s="7" t="s">
+      <c r="G100" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="H100" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="I100" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J99" s="7" t="s">
+      <c r="J100" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="K99" s="7" t="s">
+      <c r="K100" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="L99" s="7" t="s">
+      <c r="L100" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M99" s="7">
+      <c r="M100" s="7">
         <v>2.0</v>
       </c>
-      <c r="N99" s="7" t="s">
+      <c r="N100" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="O99" s="7" t="s">
+      <c r="O100" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="P99" s="8"/>
-      <c r="Q99" s="8"/>
-      <c r="R99" s="8"/>
-      <c r="S99" s="8"/>
-      <c r="T99" s="8"/>
-      <c r="U99" s="8"/>
-      <c r="V99" s="8"/>
-      <c r="W99" s="8"/>
-      <c r="X99" s="8"/>
-      <c r="Y99" s="8"/>
-      <c r="Z99" s="8"/>
-    </row>
-    <row r="100" hidden="1">
-      <c r="A100" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B100" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="C100" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D100" s="5">
-        <v>46054.0</v>
-      </c>
-      <c r="E100" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="F100" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="G100" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="H100" s="4">
-        <v>0.666666666666666</v>
-      </c>
-      <c r="I100" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J100" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K100" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="L100" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="M100" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="N100" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="O100" s="4" t="s">
-        <v>141</v>
-      </c>
+      <c r="P100" s="8"/>
+      <c r="Q100" s="8"/>
+      <c r="R100" s="8"/>
+      <c r="S100" s="8"/>
+      <c r="T100" s="8"/>
+      <c r="U100" s="8"/>
+      <c r="V100" s="8"/>
+      <c r="W100" s="8"/>
+      <c r="X100" s="8"/>
+      <c r="Y100" s="8"/>
+      <c r="Z100" s="8"/>
     </row>
     <row r="101" hidden="1">
       <c r="A101" s="4" t="s">
@@ -6043,30 +6061,30 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I101" s="4" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="J101" s="4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="K101" s="4" t="s">
-        <v>32</v>
+        <v>141</v>
       </c>
       <c r="L101" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="M101" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="N101" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="O101" s="4" t="s">
-        <v>34</v>
+        <v>141</v>
       </c>
     </row>
     <row r="102" hidden="1">
       <c r="A102" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B102" s="4">
         <v>1.0</v>
@@ -6090,25 +6108,25 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I102" s="4" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="J102" s="4" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="K102" s="4" t="s">
-        <v>143</v>
+        <v>32</v>
       </c>
       <c r="L102" s="4" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="M102" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="N102" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="O102" s="4" t="s">
-        <v>143</v>
+        <v>34</v>
       </c>
     </row>
     <row r="103" hidden="1">
@@ -6137,33 +6155,33 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I103" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="J103" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="L103" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="M103" s="4">
         <v>1.0</v>
       </c>
       <c r="N103" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="O103" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="104" hidden="1">
       <c r="A104" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B104" s="4">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="C104" s="4" t="s">
         <v>16</v>
@@ -6184,25 +6202,25 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I104" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="J104" s="4" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="K104" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L104" s="4" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="M104" s="4">
         <v>1.0</v>
       </c>
       <c r="N104" s="4" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="O104" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="105" hidden="1">
@@ -6210,7 +6228,7 @@
         <v>145</v>
       </c>
       <c r="B105" s="4">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>16</v>
@@ -6231,13 +6249,13 @@
         <v>0.666666666666666</v>
       </c>
       <c r="I105" s="4" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="J105" s="4" t="s">
         <v>25</v>
       </c>
       <c r="K105" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L105" s="4" t="s">
         <v>29</v>
@@ -6249,7 +6267,7 @@
         <v>29</v>
       </c>
       <c r="O105" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="106" hidden="1">
@@ -6257,7 +6275,7 @@
         <v>145</v>
       </c>
       <c r="B106" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>16</v>
@@ -6284,7 +6302,7 @@
         <v>25</v>
       </c>
       <c r="K106" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="L106" s="4" t="s">
         <v>29</v>
@@ -6296,108 +6314,125 @@
         <v>29</v>
       </c>
       <c r="O106" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="107" hidden="1">
+      <c r="A107" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B107" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D107" s="5">
+        <v>46054.0</v>
+      </c>
+      <c r="E107" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="F107" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="G107" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="H107" s="4">
+        <v>0.666666666666666</v>
+      </c>
+      <c r="I107" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J107" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K107" s="4" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="7" t="s">
+      <c r="L107" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="M107" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="N107" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="O107" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="B107" s="7">
+      <c r="B108" s="7">
         <v>0.0</v>
       </c>
-      <c r="C107" s="7" t="s">
+      <c r="C108" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D107" s="7" t="s">
+      <c r="D108" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E107" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="F107" s="7">
+      <c r="E108" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F108" s="7">
         <v>0.0</v>
       </c>
-      <c r="G107" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="H107" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="I107" s="7" t="s">
+      <c r="G108" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="H108" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="I108" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J107" s="7" t="s">
+      <c r="J108" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="K107" s="7" t="s">
+      <c r="K108" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="L107" s="7" t="s">
+      <c r="L108" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M107" s="7">
+      <c r="M108" s="7">
         <v>2.0</v>
       </c>
-      <c r="N107" s="7" t="s">
+      <c r="N108" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="O107" s="7" t="s">
+      <c r="O108" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="P107" s="8"/>
-      <c r="Q107" s="8"/>
-      <c r="R107" s="8"/>
-      <c r="S107" s="8"/>
-      <c r="T107" s="8"/>
-      <c r="U107" s="8"/>
-      <c r="V107" s="8"/>
-      <c r="W107" s="8"/>
-      <c r="X107" s="8"/>
-      <c r="Y107" s="8"/>
-      <c r="Z107" s="8"/>
-    </row>
-    <row r="108">
-      <c r="C108" s="9"/>
-      <c r="E108" s="9"/>
-      <c r="I108" s="8"/>
-      <c r="J108" s="8"/>
-      <c r="K108" s="8"/>
-      <c r="N108" s="8"/>
+      <c r="P108" s="8"/>
+      <c r="Q108" s="8"/>
+      <c r="R108" s="8"/>
+      <c r="S108" s="8"/>
+      <c r="T108" s="8"/>
+      <c r="U108" s="8"/>
+      <c r="V108" s="8"/>
+      <c r="W108" s="8"/>
+      <c r="X108" s="8"/>
+      <c r="Y108" s="8"/>
+      <c r="Z108" s="8"/>
     </row>
     <row r="109">
-      <c r="A109" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="B109" s="11"/>
-      <c r="C109" s="11"/>
-      <c r="D109" s="11"/>
-      <c r="E109" s="11"/>
-      <c r="F109" s="11"/>
-      <c r="G109" s="11"/>
-      <c r="H109" s="11"/>
-      <c r="I109" s="12"/>
-      <c r="J109" s="12"/>
-      <c r="K109" s="12"/>
-      <c r="L109" s="11"/>
-      <c r="M109" s="11"/>
-      <c r="N109" s="11"/>
-      <c r="O109" s="11"/>
-      <c r="P109" s="11"/>
-      <c r="Q109" s="11"/>
-      <c r="R109" s="11"/>
-      <c r="S109" s="11"/>
-      <c r="T109" s="11"/>
-      <c r="U109" s="11"/>
-      <c r="V109" s="11"/>
-      <c r="W109" s="11"/>
-      <c r="X109" s="11"/>
-      <c r="Y109" s="11"/>
-      <c r="Z109" s="11"/>
+      <c r="C109" s="9"/>
+      <c r="E109" s="9"/>
+      <c r="I109" s="8"/>
+      <c r="J109" s="8"/>
+      <c r="K109" s="8"/>
+      <c r="N109" s="8"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B110" s="11"/>
       <c r="C110" s="11"/>
@@ -6426,8 +6461,8 @@
       <c r="Z110" s="11"/>
     </row>
     <row r="111">
-      <c r="A111" s="13" t="s">
-        <v>152</v>
+      <c r="A111" s="10" t="s">
+        <v>151</v>
       </c>
       <c r="B111" s="11"/>
       <c r="C111" s="11"/>
@@ -6436,9 +6471,9 @@
       <c r="F111" s="11"/>
       <c r="G111" s="11"/>
       <c r="H111" s="11"/>
-      <c r="I111" s="11"/>
-      <c r="J111" s="11"/>
-      <c r="K111" s="11"/>
+      <c r="I111" s="12"/>
+      <c r="J111" s="12"/>
+      <c r="K111" s="12"/>
       <c r="L111" s="11"/>
       <c r="M111" s="11"/>
       <c r="N111" s="11"/>
@@ -6456,42 +6491,64 @@
       <c r="Z111" s="11"/>
     </row>
     <row r="112">
-      <c r="A112" s="10" t="s">
+      <c r="A112" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="B112" s="11"/>
+      <c r="C112" s="11"/>
+      <c r="D112" s="11"/>
+      <c r="E112" s="11"/>
+      <c r="F112" s="11"/>
+      <c r="G112" s="11"/>
+      <c r="H112" s="11"/>
+      <c r="I112" s="11"/>
+      <c r="J112" s="11"/>
+      <c r="K112" s="11"/>
+      <c r="L112" s="11"/>
+      <c r="M112" s="11"/>
+      <c r="N112" s="11"/>
+      <c r="O112" s="11"/>
+      <c r="P112" s="11"/>
+      <c r="Q112" s="11"/>
+      <c r="R112" s="11"/>
+      <c r="S112" s="11"/>
+      <c r="T112" s="11"/>
+      <c r="U112" s="11"/>
+      <c r="V112" s="11"/>
+      <c r="W112" s="11"/>
+      <c r="X112" s="11"/>
+      <c r="Y112" s="11"/>
+      <c r="Z112" s="11"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="B112" s="14"/>
-      <c r="C112" s="14"/>
-      <c r="D112" s="14"/>
-      <c r="E112" s="14"/>
-      <c r="F112" s="14"/>
-      <c r="G112" s="14"/>
-      <c r="H112" s="14"/>
-      <c r="I112" s="14"/>
-      <c r="J112" s="14"/>
-      <c r="K112" s="14"/>
-      <c r="L112" s="14"/>
-      <c r="M112" s="14"/>
-      <c r="N112" s="14"/>
-      <c r="O112" s="14"/>
-      <c r="P112" s="14"/>
-      <c r="Q112" s="14"/>
-      <c r="R112" s="14"/>
-      <c r="S112" s="14"/>
-      <c r="T112" s="14"/>
-      <c r="U112" s="14"/>
-      <c r="V112" s="14"/>
-      <c r="W112" s="14"/>
-      <c r="X112" s="14"/>
-      <c r="Y112" s="14"/>
-      <c r="Z112" s="14"/>
-    </row>
-    <row r="113">
-      <c r="C113" s="9"/>
-      <c r="E113" s="9"/>
-      <c r="I113" s="8"/>
-      <c r="J113" s="8"/>
-      <c r="K113" s="8"/>
-      <c r="N113" s="8"/>
+      <c r="B113" s="14"/>
+      <c r="C113" s="14"/>
+      <c r="D113" s="14"/>
+      <c r="E113" s="14"/>
+      <c r="F113" s="14"/>
+      <c r="G113" s="14"/>
+      <c r="H113" s="14"/>
+      <c r="I113" s="14"/>
+      <c r="J113" s="14"/>
+      <c r="K113" s="14"/>
+      <c r="L113" s="14"/>
+      <c r="M113" s="14"/>
+      <c r="N113" s="14"/>
+      <c r="O113" s="14"/>
+      <c r="P113" s="14"/>
+      <c r="Q113" s="14"/>
+      <c r="R113" s="14"/>
+      <c r="S113" s="14"/>
+      <c r="T113" s="14"/>
+      <c r="U113" s="14"/>
+      <c r="V113" s="14"/>
+      <c r="W113" s="14"/>
+      <c r="X113" s="14"/>
+      <c r="Y113" s="14"/>
+      <c r="Z113" s="14"/>
     </row>
     <row r="114">
       <c r="C114" s="9"/>
@@ -12900,6 +12957,14 @@
       <c r="J914" s="8"/>
       <c r="K914" s="8"/>
       <c r="N914" s="8"/>
+    </row>
+    <row r="915">
+      <c r="C915" s="9"/>
+      <c r="E915" s="9"/>
+      <c r="I915" s="8"/>
+      <c r="J915" s="8"/>
+      <c r="K915" s="8"/>
+      <c r="N915" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$1:$Z$107">

</xml_diff>